<commit_message>
Deploying to gh-pages from  @ 246094ef32e112c3873aa2b88aaf3884bf4a99d0 🚀
</commit_message>
<xml_diff>
--- a/en/downloads/data-excel/4.1.1.xlsx
+++ b/en/downloads/data-excel/4.1.1.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="247" uniqueCount="129">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="265" uniqueCount="138">
   <si>
     <t>Көрсөткүчтөрдүн аталышы</t>
   </si>
@@ -400,7 +400,34 @@
     <t xml:space="preserve">4.1.1 Балдардын жана жаштардын үлүшү: a) 2-/ 3-класста, b) башталгыч мектептердин бүтүрүүчүлөрү жана аз дегенде төмөнкүлөрдүн минималдуу деңгээлине жеткен c) орто мектептердин бүтүрүүчүлөрү i) сабаттуулук жана ii) эсептөө көндүмдөрүнүн, жынысы боюнча бөлүштүрүүдө                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                      </t>
   </si>
   <si>
-    <t>According to the Multiple Indicator Cluster Survey, 2018, 2023</t>
+    <t>Жынысы боюнча</t>
+  </si>
+  <si>
+    <t>По полу</t>
+  </si>
+  <si>
+    <t>By sex</t>
+  </si>
+  <si>
+    <t>Балдар</t>
+  </si>
+  <si>
+    <t>Мальчики</t>
+  </si>
+  <si>
+    <t>Boys</t>
+  </si>
+  <si>
+    <t>Кыздар</t>
+  </si>
+  <si>
+    <t>Девочки</t>
+  </si>
+  <si>
+    <t>Girls</t>
+  </si>
+  <si>
+    <t>According to the Multiple Indicator Cluster Survey, 2018, 2023.</t>
   </si>
 </sst>
 </file>
@@ -492,19 +519,19 @@
       <family val="1"/>
     </font>
     <font>
-      <i/>
-      <sz val="9"/>
-      <color theme="1"/>
-      <name val="Times New Roman"/>
-      <family val="1"/>
-    </font>
-    <font>
       <b/>
       <sz val="10"/>
       <color theme="1"/>
       <name val="Times New Roman"/>
       <family val="1"/>
       <charset val="204"/>
+    </font>
+    <font>
+      <i/>
+      <sz val="8"/>
+      <color theme="1"/>
+      <name val="Times New Roman"/>
+      <family val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -643,11 +670,11 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -957,7 +984,7 @@
   <sheetPr codeName="Лист1">
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:F240"/>
+  <dimension ref="A1:F246"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="42.7109375" customWidth="1"/>
@@ -966,7 +993,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="84.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="32" t="s">
+      <c r="A1" s="31" t="s">
         <v>127</v>
       </c>
       <c r="B1" s="5" t="s">
@@ -980,13 +1007,13 @@
       <c r="F1" s="1"/>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A2" s="31" t="s">
+      <c r="A2" s="32" t="s">
         <v>120</v>
       </c>
-      <c r="B2" s="31" t="s">
+      <c r="B2" s="32" t="s">
         <v>121</v>
       </c>
-      <c r="C2" s="31" t="s">
+      <c r="C2" s="32" t="s">
         <v>122</v>
       </c>
       <c r="D2" s="1"/>
@@ -1087,436 +1114,437 @@
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A9" s="20" t="s">
+        <v>128</v>
+      </c>
+      <c r="B9" s="10" t="s">
+        <v>129</v>
+      </c>
+      <c r="C9" s="10" t="s">
+        <v>130</v>
+      </c>
+      <c r="F9" s="1"/>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A10" s="21" t="s">
+        <v>131</v>
+      </c>
+      <c r="B10" s="9" t="s">
+        <v>132</v>
+      </c>
+      <c r="C10" s="15" t="s">
+        <v>133</v>
+      </c>
+      <c r="D10" s="6">
+        <v>55.8</v>
+      </c>
+      <c r="E10" s="6">
+        <v>66.900000000000006</v>
+      </c>
+      <c r="F10" s="1"/>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A11" s="21" t="s">
+        <v>134</v>
+      </c>
+      <c r="B11" s="9" t="s">
+        <v>135</v>
+      </c>
+      <c r="C11" s="15" t="s">
+        <v>136</v>
+      </c>
+      <c r="D11" s="6">
+        <v>60.1</v>
+      </c>
+      <c r="E11" s="6">
+        <v>70.099999999999994</v>
+      </c>
+      <c r="F11" s="1"/>
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A12" s="20" t="s">
         <v>84</v>
       </c>
-      <c r="B9" s="10" t="s">
+      <c r="B12" s="10" t="s">
         <v>50</v>
       </c>
-      <c r="C9" s="10" t="s">
+      <c r="C12" s="10" t="s">
         <v>54</v>
       </c>
-      <c r="D9" s="6"/>
-      <c r="E9" s="6"/>
-      <c r="F9" s="1"/>
-    </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A10" s="22" t="s">
-        <v>75</v>
-      </c>
-      <c r="B10" s="9" t="s">
-        <v>4</v>
-      </c>
-      <c r="C10" s="15" t="s">
-        <v>35</v>
-      </c>
-      <c r="D10" s="6">
-        <v>66</v>
-      </c>
-      <c r="E10" s="6">
-        <v>81.099999999999994</v>
-      </c>
-      <c r="F10" s="1"/>
-    </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A11" s="22" t="s">
-        <v>76</v>
-      </c>
-      <c r="B11" s="9" t="s">
-        <v>5</v>
-      </c>
-      <c r="C11" s="19" t="s">
-        <v>36</v>
-      </c>
-      <c r="D11" s="6">
-        <v>50</v>
-      </c>
-      <c r="E11" s="6">
-        <v>76.5</v>
-      </c>
-      <c r="F11" s="1"/>
-    </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A12" s="22" t="s">
-        <v>77</v>
-      </c>
-      <c r="B12" s="9" t="s">
-        <v>6</v>
-      </c>
-      <c r="C12" s="19" t="s">
-        <v>37</v>
-      </c>
-      <c r="D12" s="6">
-        <v>65</v>
-      </c>
-      <c r="E12" s="6">
-        <v>84.4</v>
-      </c>
+      <c r="D12" s="6"/>
+      <c r="E12" s="6"/>
       <c r="F12" s="1"/>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A13" s="22" t="s">
-        <v>78</v>
+        <v>75</v>
       </c>
       <c r="B13" s="9" t="s">
-        <v>7</v>
-      </c>
-      <c r="C13" s="19" t="s">
-        <v>38</v>
-      </c>
-      <c r="D13" s="8">
-        <v>39</v>
-      </c>
-      <c r="E13" s="8">
-        <v>58.2</v>
+        <v>4</v>
+      </c>
+      <c r="C13" s="15" t="s">
+        <v>35</v>
+      </c>
+      <c r="D13" s="6">
+        <v>66</v>
+      </c>
+      <c r="E13" s="6">
+        <v>81.099999999999994</v>
       </c>
       <c r="F13" s="1"/>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A14" s="22" t="s">
-        <v>79</v>
+        <v>76</v>
       </c>
       <c r="B14" s="9" t="s">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="C14" s="19" t="s">
-        <v>39</v>
-      </c>
-      <c r="D14" s="8">
-        <v>55</v>
-      </c>
-      <c r="E14" s="8">
-        <v>56.6</v>
+        <v>36</v>
+      </c>
+      <c r="D14" s="6">
+        <v>50</v>
+      </c>
+      <c r="E14" s="6">
+        <v>76.5</v>
       </c>
       <c r="F14" s="1"/>
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A15" s="22" t="s">
-        <v>80</v>
+        <v>77</v>
       </c>
       <c r="B15" s="9" t="s">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="C15" s="19" t="s">
-        <v>40</v>
-      </c>
-      <c r="D15" s="1">
+        <v>37</v>
+      </c>
+      <c r="D15" s="6">
         <v>65</v>
       </c>
-      <c r="E15" s="1">
-        <v>75.5</v>
+      <c r="E15" s="6">
+        <v>84.4</v>
       </c>
       <c r="F15" s="1"/>
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A16" s="22" t="s">
+        <v>78</v>
+      </c>
+      <c r="B16" s="9" t="s">
+        <v>7</v>
+      </c>
+      <c r="C16" s="19" t="s">
+        <v>38</v>
+      </c>
+      <c r="D16" s="8">
+        <v>39</v>
+      </c>
+      <c r="E16" s="8">
+        <v>58.2</v>
+      </c>
+      <c r="F16" s="1"/>
+    </row>
+    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A17" s="22" t="s">
+        <v>79</v>
+      </c>
+      <c r="B17" s="9" t="s">
+        <v>8</v>
+      </c>
+      <c r="C17" s="19" t="s">
+        <v>39</v>
+      </c>
+      <c r="D17" s="8">
+        <v>55</v>
+      </c>
+      <c r="E17" s="8">
+        <v>56.6</v>
+      </c>
+      <c r="F17" s="1"/>
+    </row>
+    <row r="18" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A18" s="22" t="s">
+        <v>80</v>
+      </c>
+      <c r="B18" s="9" t="s">
+        <v>9</v>
+      </c>
+      <c r="C18" s="19" t="s">
+        <v>40</v>
+      </c>
+      <c r="D18" s="1">
+        <v>65</v>
+      </c>
+      <c r="E18" s="1">
+        <v>75.5</v>
+      </c>
+      <c r="F18" s="1"/>
+    </row>
+    <row r="19" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A19" s="22" t="s">
         <v>81</v>
       </c>
-      <c r="B16" s="9" t="s">
+      <c r="B19" s="9" t="s">
         <v>10</v>
       </c>
-      <c r="C16" s="19" t="s">
+      <c r="C19" s="19" t="s">
         <v>41</v>
       </c>
-      <c r="D16" s="1">
+      <c r="D19" s="1">
         <v>49</v>
       </c>
-      <c r="E16" s="1">
+      <c r="E19" s="1">
         <v>58.1</v>
       </c>
-      <c r="F16" s="1"/>
-    </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A17" s="23" t="s">
+      <c r="F19" s="1"/>
+    </row>
+    <row r="20" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A20" s="23" t="s">
         <v>82</v>
       </c>
-      <c r="B17" s="9" t="s">
+      <c r="B20" s="9" t="s">
         <v>11</v>
       </c>
-      <c r="C17" s="19" t="s">
+      <c r="C20" s="19" t="s">
         <v>42</v>
       </c>
-      <c r="D17" s="1">
+      <c r="D20" s="1">
         <v>74</v>
       </c>
-      <c r="E17" s="1">
+      <c r="E20" s="1">
         <v>85.7</v>
       </c>
-      <c r="F17" s="1"/>
-    </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A18" s="23" t="s">
+      <c r="F20" s="1"/>
+    </row>
+    <row r="21" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A21" s="23" t="s">
         <v>83</v>
       </c>
-      <c r="B18" s="9" t="s">
+      <c r="B21" s="9" t="s">
         <v>12</v>
       </c>
-      <c r="C18" s="15" t="s">
+      <c r="C21" s="15" t="s">
         <v>43</v>
       </c>
-      <c r="D18" s="1">
+      <c r="D21" s="1">
         <v>72</v>
       </c>
-      <c r="E18" s="1">
+      <c r="E21" s="1">
         <v>57</v>
       </c>
-      <c r="F18" s="1"/>
-    </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A19" s="10" t="s">
+      <c r="F21" s="1"/>
+    </row>
+    <row r="22" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A22" s="10" t="s">
         <v>101</v>
       </c>
-      <c r="B19" s="10" t="s">
+      <c r="B22" s="10" t="s">
         <v>51</v>
       </c>
-      <c r="C19" s="10" t="s">
+      <c r="C22" s="10" t="s">
         <v>55</v>
       </c>
-      <c r="D19" s="6">
+      <c r="D22" s="6">
         <v>47.4</v>
       </c>
-      <c r="E19" s="6">
+      <c r="E22" s="6">
         <v>53.7</v>
       </c>
-      <c r="F19" s="1"/>
-    </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A20" s="1" t="s">
+      <c r="F22" s="1"/>
+    </row>
+    <row r="23" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A23" s="1" t="s">
         <v>85</v>
       </c>
-      <c r="B20" s="9" t="s">
+      <c r="B23" s="9" t="s">
         <v>15</v>
       </c>
-      <c r="C20" s="9" t="s">
+      <c r="C23" s="9" t="s">
         <v>44</v>
       </c>
-      <c r="D20" s="13">
+      <c r="D23" s="13">
         <v>43</v>
       </c>
-      <c r="E20" s="13">
+      <c r="E23" s="13">
         <v>46.6</v>
       </c>
-      <c r="F20" s="1"/>
-    </row>
-    <row r="21" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A21" s="1" t="s">
+      <c r="F23" s="1"/>
+    </row>
+    <row r="24" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A24" s="1" t="s">
         <v>86</v>
       </c>
-      <c r="B21" s="12" t="s">
+      <c r="B24" s="12" t="s">
         <v>16</v>
       </c>
-      <c r="C21" s="9" t="s">
+      <c r="C24" s="9" t="s">
         <v>45</v>
       </c>
-      <c r="D21" s="1">
+      <c r="D24" s="1">
         <v>52.3</v>
       </c>
-      <c r="E21" s="1">
+      <c r="E24" s="1">
         <v>60.5</v>
       </c>
-      <c r="F21" s="1"/>
-    </row>
-    <row r="22" spans="1:6" s="28" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A22" s="10" t="s">
+      <c r="F24" s="1"/>
+    </row>
+    <row r="25" spans="1:6" s="28" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A25" s="10" t="s">
         <v>109</v>
       </c>
-      <c r="B22" s="10" t="s">
+      <c r="B25" s="10" t="s">
         <v>110</v>
       </c>
-      <c r="C22" s="10" t="s">
+      <c r="C25" s="10" t="s">
         <v>108</v>
       </c>
-      <c r="D22" s="6">
+      <c r="D25" s="6">
         <v>58.1</v>
       </c>
-      <c r="E22" s="6">
+      <c r="E25" s="6">
         <v>67.599999999999994</v>
       </c>
-      <c r="F22" s="27"/>
-    </row>
-    <row r="23" spans="1:6" s="28" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A23" s="10" t="s">
+      <c r="F25" s="27"/>
+    </row>
+    <row r="26" spans="1:6" s="28" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A26" s="10" t="s">
         <v>112</v>
       </c>
-      <c r="B23" s="10" t="s">
+      <c r="B26" s="10" t="s">
         <v>111</v>
       </c>
-      <c r="C23" s="10" t="s">
+      <c r="C26" s="10" t="s">
         <v>113</v>
       </c>
-      <c r="D23" s="6">
+      <c r="D26" s="6">
         <v>78.599999999999994</v>
       </c>
-      <c r="E23" s="6">
+      <c r="E26" s="6">
         <v>89.1</v>
       </c>
-      <c r="F23" s="27"/>
-    </row>
-    <row r="24" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A24" s="20" t="s">
+      <c r="F26" s="27"/>
+    </row>
+    <row r="27" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A27" s="20" t="s">
         <v>91</v>
       </c>
-      <c r="B24" s="14" t="s">
+      <c r="B27" s="14" t="s">
         <v>52</v>
       </c>
-      <c r="C24" s="14" t="s">
+      <c r="C27" s="14" t="s">
         <v>56</v>
       </c>
-      <c r="D24" s="1"/>
-      <c r="E24" s="1"/>
-      <c r="F24" s="1"/>
-    </row>
-    <row r="25" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A25" s="21" t="s">
-        <v>87</v>
-      </c>
-      <c r="B25" s="15" t="s">
-        <v>17</v>
-      </c>
-      <c r="C25" s="15" t="s">
-        <v>58</v>
-      </c>
-      <c r="D25" s="6" t="s">
-        <v>22</v>
-      </c>
-      <c r="E25" s="6" t="s">
-        <v>22</v>
-      </c>
-      <c r="F25" s="1"/>
-    </row>
-    <row r="26" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A26" s="21" t="s">
-        <v>88</v>
-      </c>
-      <c r="B26" s="15" t="s">
-        <v>18</v>
-      </c>
-      <c r="C26" s="15" t="s">
-        <v>59</v>
-      </c>
-      <c r="D26" s="1">
-        <v>51.7</v>
-      </c>
-      <c r="E26" s="1">
-        <v>51.6</v>
-      </c>
-      <c r="F26" s="1"/>
-    </row>
-    <row r="27" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A27" s="21" t="s">
-        <v>102</v>
-      </c>
-      <c r="B27" s="15" t="s">
-        <v>19</v>
-      </c>
-      <c r="C27" s="15" t="s">
-        <v>60</v>
-      </c>
-      <c r="D27" s="1">
-        <v>55.2</v>
-      </c>
-      <c r="E27" s="1">
-        <v>66.8</v>
-      </c>
+      <c r="D27" s="1"/>
+      <c r="E27" s="1"/>
       <c r="F27" s="1"/>
     </row>
     <row r="28" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A28" s="21" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="B28" s="15" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="C28" s="15" t="s">
-        <v>61</v>
-      </c>
-      <c r="D28" s="1">
-        <v>59.6</v>
-      </c>
-      <c r="E28" s="1">
-        <v>73.400000000000006</v>
+        <v>58</v>
+      </c>
+      <c r="D28" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="E28" s="6" t="s">
+        <v>22</v>
       </c>
       <c r="F28" s="1"/>
     </row>
     <row r="29" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A29" s="21" t="s">
+        <v>88</v>
+      </c>
+      <c r="B29" s="15" t="s">
+        <v>18</v>
+      </c>
+      <c r="C29" s="15" t="s">
+        <v>59</v>
+      </c>
+      <c r="D29" s="1">
+        <v>51.7</v>
+      </c>
+      <c r="E29" s="1">
+        <v>51.6</v>
+      </c>
+      <c r="F29" s="1"/>
+    </row>
+    <row r="30" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A30" s="21" t="s">
+        <v>102</v>
+      </c>
+      <c r="B30" s="15" t="s">
+        <v>19</v>
+      </c>
+      <c r="C30" s="15" t="s">
+        <v>60</v>
+      </c>
+      <c r="D30" s="1">
+        <v>55.2</v>
+      </c>
+      <c r="E30" s="1">
+        <v>66.8</v>
+      </c>
+      <c r="F30" s="1"/>
+    </row>
+    <row r="31" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A31" s="21" t="s">
+        <v>89</v>
+      </c>
+      <c r="B31" s="15" t="s">
+        <v>20</v>
+      </c>
+      <c r="C31" s="15" t="s">
+        <v>61</v>
+      </c>
+      <c r="D31" s="1">
+        <v>59.6</v>
+      </c>
+      <c r="E31" s="1">
+        <v>73.400000000000006</v>
+      </c>
+      <c r="F31" s="1"/>
+    </row>
+    <row r="32" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A32" s="21" t="s">
         <v>90</v>
       </c>
-      <c r="B29" s="15" t="s">
+      <c r="B32" s="15" t="s">
         <v>21</v>
       </c>
-      <c r="C29" s="15" t="s">
+      <c r="C32" s="15" t="s">
         <v>62</v>
       </c>
-      <c r="D29" s="13">
+      <c r="D32" s="13">
         <v>64</v>
       </c>
-      <c r="E29" s="13">
+      <c r="E32" s="13">
         <v>72.599999999999994</v>
       </c>
-      <c r="F29" s="1"/>
-    </row>
-    <row r="30" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A30" s="27" t="s">
+      <c r="F32" s="1"/>
+    </row>
+    <row r="33" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A33" s="27" t="s">
         <v>106</v>
       </c>
-      <c r="B30" s="14" t="s">
+      <c r="B33" s="14" t="s">
         <v>23</v>
       </c>
-      <c r="C30" s="14" t="s">
+      <c r="C33" s="14" t="s">
         <v>46</v>
       </c>
-      <c r="D30" s="1"/>
-      <c r="E30" s="1"/>
-      <c r="F30" s="1"/>
-    </row>
-    <row r="31" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A31" s="1" t="s">
-        <v>92</v>
-      </c>
-      <c r="B31" s="9" t="s">
-        <v>24</v>
-      </c>
-      <c r="C31" s="9" t="s">
-        <v>63</v>
-      </c>
-      <c r="D31" s="1">
-        <v>42.3</v>
-      </c>
-      <c r="E31" s="1">
-        <v>70.099999999999994</v>
-      </c>
-      <c r="F31" s="1"/>
-    </row>
-    <row r="32" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A32" s="1" t="s">
-        <v>93</v>
-      </c>
-      <c r="B32" s="9" t="s">
-        <v>25</v>
-      </c>
-      <c r="C32" s="9" t="s">
-        <v>64</v>
-      </c>
-      <c r="D32" s="1">
-        <v>59.4</v>
-      </c>
-      <c r="E32" s="1">
-        <v>68.400000000000006</v>
-      </c>
-      <c r="F32" s="1"/>
-    </row>
-    <row r="33" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A33" s="27" t="s">
-        <v>107</v>
-      </c>
-      <c r="B33" s="14" t="s">
-        <v>26</v>
-      </c>
-      <c r="C33" s="14" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="34" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="D33" s="1"/>
+      <c r="E33" s="1"/>
+      <c r="F33" s="1"/>
+    </row>
+    <row r="34" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A34" s="1" t="s">
         <v>92</v>
       </c>
@@ -1527,13 +1555,14 @@
         <v>63</v>
       </c>
       <c r="D34" s="1">
-        <v>43.4</v>
-      </c>
-      <c r="E34" s="6" t="s">
-        <v>123</v>
-      </c>
-    </row>
-    <row r="35" spans="1:5" x14ac:dyDescent="0.25">
+        <v>42.3</v>
+      </c>
+      <c r="E34" s="1">
+        <v>70.099999999999994</v>
+      </c>
+      <c r="F34" s="1"/>
+    </row>
+    <row r="35" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A35" s="1" t="s">
         <v>93</v>
       </c>
@@ -1544,812 +1573,882 @@
         <v>64</v>
       </c>
       <c r="D35" s="1">
+        <v>59.4</v>
+      </c>
+      <c r="E35" s="1">
+        <v>68.400000000000006</v>
+      </c>
+      <c r="F35" s="1"/>
+    </row>
+    <row r="36" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A36" s="27" t="s">
+        <v>107</v>
+      </c>
+      <c r="B36" s="14" t="s">
+        <v>26</v>
+      </c>
+      <c r="C36" s="14" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="37" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A37" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="B37" s="9" t="s">
+        <v>24</v>
+      </c>
+      <c r="C37" s="9" t="s">
+        <v>63</v>
+      </c>
+      <c r="D37" s="1">
+        <v>43.4</v>
+      </c>
+      <c r="E37" s="6" t="s">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="38" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A38" s="1" t="s">
+        <v>93</v>
+      </c>
+      <c r="B38" s="9" t="s">
+        <v>25</v>
+      </c>
+      <c r="C38" s="9" t="s">
+        <v>64</v>
+      </c>
+      <c r="D38" s="1">
         <v>57.8</v>
       </c>
-      <c r="E35" s="1">
+      <c r="E38" s="1">
         <v>66.8</v>
       </c>
     </row>
-    <row r="36" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A36" s="1" t="s">
+    <row r="39" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A39" s="1" t="s">
         <v>94</v>
       </c>
-      <c r="B36" s="9" t="s">
+      <c r="B39" s="9" t="s">
         <v>27</v>
       </c>
-      <c r="C36" s="9" t="s">
+      <c r="C39" s="9" t="s">
         <v>65</v>
       </c>
-      <c r="D36" s="13">
+      <c r="D39" s="13">
         <v>61</v>
       </c>
-      <c r="E36" s="13"/>
-    </row>
-    <row r="37" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A37" s="14" t="s">
+      <c r="E39" s="13"/>
+    </row>
+    <row r="40" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A40" s="14" t="s">
         <v>103</v>
       </c>
-      <c r="B37" s="14" t="s">
+      <c r="B40" s="14" t="s">
         <v>53</v>
       </c>
-      <c r="C37" s="14" t="s">
+      <c r="C40" s="14" t="s">
         <v>57</v>
       </c>
     </row>
-    <row r="38" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A38" s="24" t="s">
+    <row r="41" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A41" s="24" t="s">
         <v>95</v>
       </c>
-      <c r="B38" s="15" t="s">
+      <c r="B41" s="15" t="s">
         <v>28</v>
       </c>
-      <c r="C38" s="15" t="s">
+      <c r="C41" s="15" t="s">
         <v>66</v>
       </c>
-      <c r="D38" s="1">
+      <c r="D41" s="1">
         <v>53.1</v>
       </c>
-      <c r="E38" s="1">
+      <c r="E41" s="1">
         <v>59.5</v>
       </c>
     </row>
-    <row r="39" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A39" s="24" t="s">
+    <row r="42" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A42" s="24" t="s">
         <v>96</v>
       </c>
-      <c r="B39" s="15" t="s">
+      <c r="B42" s="15" t="s">
         <v>29</v>
       </c>
-      <c r="C39" s="15" t="s">
+      <c r="C42" s="15" t="s">
         <v>67</v>
       </c>
-      <c r="D39" s="1">
+      <c r="D42" s="1">
         <v>52.1</v>
       </c>
-      <c r="E39" s="1">
+      <c r="E42" s="1">
         <v>67.3</v>
       </c>
     </row>
-    <row r="40" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A40" s="24" t="s">
+    <row r="43" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A43" s="24" t="s">
         <v>97</v>
       </c>
-      <c r="B40" s="15" t="s">
+      <c r="B43" s="15" t="s">
         <v>30</v>
       </c>
-      <c r="C40" s="15" t="s">
+      <c r="C43" s="15" t="s">
         <v>68</v>
       </c>
-      <c r="D40" s="13">
+      <c r="D43" s="13">
         <v>52.9</v>
       </c>
-      <c r="E40" s="13">
+      <c r="E43" s="13">
         <v>67</v>
       </c>
     </row>
-    <row r="41" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A41" s="24" t="s">
+    <row r="44" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A44" s="24" t="s">
         <v>98</v>
       </c>
-      <c r="B41" s="15" t="s">
+      <c r="B44" s="15" t="s">
         <v>31</v>
       </c>
-      <c r="C41" s="15" t="s">
+      <c r="C44" s="15" t="s">
         <v>69</v>
       </c>
-      <c r="D41" s="1">
+      <c r="D44" s="1">
         <v>60.3</v>
       </c>
-      <c r="E41" s="1">
+      <c r="E44" s="1">
         <v>73</v>
       </c>
     </row>
-    <row r="42" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A42" s="25" t="s">
+    <row r="45" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A45" s="25" t="s">
         <v>99</v>
       </c>
-      <c r="B42" s="15" t="s">
+      <c r="B45" s="15" t="s">
         <v>32</v>
       </c>
-      <c r="C42" s="15" t="s">
+      <c r="C45" s="15" t="s">
         <v>70</v>
       </c>
-      <c r="D42" s="1">
+      <c r="D45" s="1">
         <v>76.599999999999994</v>
       </c>
-      <c r="E42" s="1">
+      <c r="E45" s="1">
         <v>78.2</v>
       </c>
     </row>
-    <row r="43" spans="1:5" ht="36" x14ac:dyDescent="0.25">
-      <c r="A43" s="30" t="s">
+    <row r="46" spans="1:6" ht="36" x14ac:dyDescent="0.25">
+      <c r="A46" s="30" t="s">
         <v>115</v>
       </c>
-      <c r="B43" s="11" t="s">
+      <c r="B46" s="11" t="s">
         <v>114</v>
       </c>
-      <c r="C43" s="30" t="s">
+      <c r="C46" s="30" t="s">
         <v>116</v>
       </c>
-      <c r="D43" s="6">
+      <c r="D46" s="6">
         <v>51.3</v>
       </c>
-      <c r="E43" s="6">
+      <c r="E46" s="6">
         <v>57</v>
       </c>
     </row>
-    <row r="44" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A44" s="20" t="s">
+    <row r="47" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A47" s="20" t="s">
         <v>72</v>
       </c>
-      <c r="B44" s="10" t="s">
+      <c r="B47" s="10" t="s">
         <v>48</v>
       </c>
-      <c r="C44" s="10" t="s">
+      <c r="C47" s="10" t="s">
         <v>49</v>
       </c>
     </row>
-    <row r="45" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A45" s="21" t="s">
+    <row r="48" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A48" s="21" t="s">
         <v>73</v>
       </c>
-      <c r="B45" s="9" t="s">
+      <c r="B48" s="9" t="s">
         <v>13</v>
       </c>
-      <c r="C45" s="15" t="s">
+      <c r="C48" s="15" t="s">
         <v>33</v>
       </c>
-      <c r="D45" s="13">
+      <c r="D48" s="13">
         <v>56.4</v>
       </c>
-      <c r="E45" s="13">
+      <c r="E48" s="13">
         <v>62.7</v>
       </c>
     </row>
-    <row r="46" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A46" s="21" t="s">
+    <row r="49" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A49" s="21" t="s">
         <v>74</v>
       </c>
-      <c r="B46" s="9" t="s">
+      <c r="B49" s="9" t="s">
         <v>14</v>
       </c>
-      <c r="C46" s="15" t="s">
+      <c r="C49" s="15" t="s">
         <v>34</v>
       </c>
-      <c r="D46" s="13">
+      <c r="D49" s="13">
         <v>49</v>
       </c>
-      <c r="E46" s="13">
+      <c r="E49" s="13">
         <v>54.6</v>
       </c>
     </row>
-    <row r="47" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A47" s="20" t="s">
+    <row r="50" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A50" s="20" t="s">
+        <v>128</v>
+      </c>
+      <c r="B50" s="10" t="s">
+        <v>129</v>
+      </c>
+      <c r="C50" s="10" t="s">
+        <v>130</v>
+      </c>
+      <c r="F50" s="1"/>
+    </row>
+    <row r="51" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A51" s="21" t="s">
+        <v>131</v>
+      </c>
+      <c r="B51" s="9" t="s">
+        <v>132</v>
+      </c>
+      <c r="C51" s="15" t="s">
+        <v>133</v>
+      </c>
+      <c r="D51" s="6">
+        <v>49.3</v>
+      </c>
+      <c r="E51" s="6">
+        <v>57</v>
+      </c>
+      <c r="F51" s="1"/>
+    </row>
+    <row r="52" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A52" s="21" t="s">
+        <v>134</v>
+      </c>
+      <c r="B52" s="9" t="s">
+        <v>135</v>
+      </c>
+      <c r="C52" s="15" t="s">
+        <v>136</v>
+      </c>
+      <c r="D52" s="6">
+        <v>53.5</v>
+      </c>
+      <c r="E52" s="6">
+        <v>56.9</v>
+      </c>
+      <c r="F52" s="1"/>
+    </row>
+    <row r="53" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A53" s="20" t="s">
         <v>84</v>
       </c>
-      <c r="B47" s="10" t="s">
+      <c r="B53" s="10" t="s">
         <v>50</v>
       </c>
-      <c r="C47" s="10" t="s">
+      <c r="C53" s="10" t="s">
         <v>54</v>
       </c>
-      <c r="D47" s="13"/>
-      <c r="E47" s="13"/>
-    </row>
-    <row r="48" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A48" s="22" t="s">
+      <c r="D53" s="13"/>
+      <c r="E53" s="13"/>
+    </row>
+    <row r="54" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A54" s="22" t="s">
         <v>75</v>
       </c>
-      <c r="B48" s="9" t="s">
+      <c r="B54" s="9" t="s">
         <v>4</v>
       </c>
-      <c r="C48" s="15" t="s">
+      <c r="C54" s="15" t="s">
         <v>35</v>
       </c>
-      <c r="D48" s="13">
+      <c r="D54" s="13">
         <v>66.7</v>
       </c>
-      <c r="E48" s="13">
+      <c r="E54" s="13">
         <v>73.900000000000006</v>
       </c>
     </row>
-    <row r="49" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A49" s="22" t="s">
+    <row r="55" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A55" s="22" t="s">
         <v>76</v>
       </c>
-      <c r="B49" s="9" t="s">
+      <c r="B55" s="9" t="s">
         <v>5</v>
       </c>
-      <c r="C49" s="19" t="s">
+      <c r="C55" s="19" t="s">
         <v>36</v>
       </c>
-      <c r="D49" s="13">
+      <c r="D55" s="13">
         <v>42.9</v>
       </c>
-      <c r="E49" s="13">
+      <c r="E55" s="13">
         <v>61.6</v>
       </c>
     </row>
-    <row r="50" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A50" s="22" t="s">
+    <row r="56" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A56" s="22" t="s">
         <v>77</v>
       </c>
-      <c r="B50" s="9" t="s">
+      <c r="B56" s="9" t="s">
         <v>6</v>
       </c>
-      <c r="C50" s="19" t="s">
+      <c r="C56" s="19" t="s">
         <v>37</v>
       </c>
-      <c r="D50" s="18">
+      <c r="D56" s="18">
         <v>54.5</v>
       </c>
-      <c r="E50" s="18">
+      <c r="E56" s="18">
         <v>69.599999999999994</v>
       </c>
     </row>
-    <row r="51" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A51" s="22" t="s">
+    <row r="57" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A57" s="22" t="s">
         <v>78</v>
       </c>
-      <c r="B51" s="9" t="s">
+      <c r="B57" s="9" t="s">
         <v>7</v>
       </c>
-      <c r="C51" s="19" t="s">
+      <c r="C57" s="19" t="s">
         <v>38</v>
       </c>
-      <c r="D51" s="13">
+      <c r="D57" s="13">
         <v>41.4</v>
       </c>
-      <c r="E51" s="13">
+      <c r="E57" s="13">
         <v>50.9</v>
       </c>
     </row>
-    <row r="52" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A52" s="22" t="s">
+    <row r="58" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A58" s="22" t="s">
         <v>79</v>
       </c>
-      <c r="B52" s="9" t="s">
+      <c r="B58" s="9" t="s">
         <v>8</v>
       </c>
-      <c r="C52" s="19" t="s">
+      <c r="C58" s="19" t="s">
         <v>39</v>
       </c>
-      <c r="D52" s="13">
+      <c r="D58" s="13">
         <v>49.2</v>
       </c>
-      <c r="E52" s="13">
+      <c r="E58" s="13">
         <v>51.2</v>
       </c>
     </row>
-    <row r="53" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A53" s="22" t="s">
+    <row r="59" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A59" s="22" t="s">
         <v>80</v>
       </c>
-      <c r="B53" s="9" t="s">
+      <c r="B59" s="9" t="s">
         <v>9</v>
       </c>
-      <c r="C53" s="19" t="s">
+      <c r="C59" s="19" t="s">
         <v>40</v>
       </c>
-      <c r="D53" s="13">
+      <c r="D59" s="13">
         <v>49.3</v>
       </c>
-      <c r="E53" s="13">
+      <c r="E59" s="13">
         <v>65.3</v>
       </c>
     </row>
-    <row r="54" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A54" s="22" t="s">
+    <row r="60" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A60" s="22" t="s">
         <v>81</v>
       </c>
-      <c r="B54" s="9" t="s">
+      <c r="B60" s="9" t="s">
         <v>10</v>
       </c>
-      <c r="C54" s="19" t="s">
+      <c r="C60" s="19" t="s">
         <v>41</v>
       </c>
-      <c r="D54" s="13">
+      <c r="D60" s="13">
         <v>46</v>
       </c>
-      <c r="E54" s="13">
+      <c r="E60" s="13">
         <v>37.799999999999997</v>
       </c>
     </row>
-    <row r="55" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A55" s="23" t="s">
+    <row r="61" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A61" s="23" t="s">
         <v>82</v>
       </c>
-      <c r="B55" s="9" t="s">
+      <c r="B61" s="9" t="s">
         <v>11</v>
       </c>
-      <c r="C55" s="19" t="s">
+      <c r="C61" s="19" t="s">
         <v>42</v>
       </c>
-      <c r="D55" s="13">
+      <c r="D61" s="13">
         <v>64.5</v>
       </c>
-      <c r="E55" s="13">
+      <c r="E61" s="13">
         <v>73.8</v>
       </c>
     </row>
-    <row r="56" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A56" s="23" t="s">
+    <row r="62" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A62" s="23" t="s">
         <v>83</v>
       </c>
-      <c r="B56" s="9" t="s">
+      <c r="B62" s="9" t="s">
         <v>12</v>
       </c>
-      <c r="C56" s="15" t="s">
+      <c r="C62" s="15" t="s">
         <v>43</v>
       </c>
-      <c r="D56" s="18">
+      <c r="D62" s="18">
         <v>54.2</v>
       </c>
-      <c r="E56" s="18">
+      <c r="E62" s="18">
         <v>51.5</v>
       </c>
     </row>
-    <row r="57" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A57" s="10" t="s">
+    <row r="63" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A63" s="10" t="s">
         <v>101</v>
       </c>
-      <c r="B57" s="10" t="s">
+      <c r="B63" s="10" t="s">
         <v>51</v>
       </c>
-      <c r="C57" s="10" t="s">
+      <c r="C63" s="10" t="s">
         <v>55</v>
       </c>
-      <c r="D57" s="13">
+      <c r="D63" s="13">
         <v>41.8</v>
       </c>
-      <c r="E57" s="13">
+      <c r="E63" s="13">
         <v>41.9</v>
       </c>
     </row>
-    <row r="58" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A58" s="1" t="s">
+    <row r="64" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A64" s="1" t="s">
         <v>85</v>
       </c>
-      <c r="B58" s="9" t="s">
+      <c r="B64" s="9" t="s">
         <v>15</v>
       </c>
-      <c r="C58" s="9" t="s">
+      <c r="C64" s="9" t="s">
         <v>44</v>
       </c>
-      <c r="D58" s="13">
+      <c r="D64" s="13">
         <v>32.6</v>
       </c>
-      <c r="E58" s="13">
+      <c r="E64" s="13">
         <v>34.1</v>
       </c>
     </row>
-    <row r="59" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A59" s="1" t="s">
+    <row r="65" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A65" s="1" t="s">
         <v>86</v>
       </c>
-      <c r="B59" s="12" t="s">
+      <c r="B65" s="12" t="s">
         <v>16</v>
       </c>
-      <c r="C59" s="9" t="s">
+      <c r="C65" s="9" t="s">
         <v>45</v>
       </c>
-      <c r="D59" s="13">
+      <c r="D65" s="13">
         <v>52</v>
       </c>
-      <c r="E59" s="13">
+      <c r="E65" s="13">
         <v>49.4</v>
       </c>
     </row>
-    <row r="60" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A60" s="10" t="s">
+    <row r="66" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A66" s="10" t="s">
         <v>109</v>
       </c>
-      <c r="B60" s="10" t="s">
+      <c r="B66" s="10" t="s">
         <v>110</v>
       </c>
-      <c r="C60" s="10" t="s">
+      <c r="C66" s="10" t="s">
         <v>108</v>
       </c>
-      <c r="D60" s="13">
+      <c r="D66" s="13">
         <v>54.9</v>
       </c>
-      <c r="E60" s="13">
+      <c r="E66" s="13">
         <v>58</v>
       </c>
     </row>
-    <row r="61" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A61" s="10" t="s">
+    <row r="67" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A67" s="10" t="s">
         <v>112</v>
       </c>
-      <c r="B61" s="10" t="s">
+      <c r="B67" s="10" t="s">
         <v>111</v>
       </c>
-      <c r="C61" s="10" t="s">
+      <c r="C67" s="10" t="s">
         <v>113</v>
       </c>
-      <c r="D61" s="13">
+      <c r="D67" s="13">
         <v>67.8</v>
       </c>
-      <c r="E61" s="13">
+      <c r="E67" s="13">
         <v>80.099999999999994</v>
       </c>
     </row>
-    <row r="62" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A62" s="20" t="s">
+    <row r="68" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A68" s="20" t="s">
         <v>91</v>
       </c>
-      <c r="B62" s="14" t="s">
+      <c r="B68" s="14" t="s">
         <v>52</v>
       </c>
-      <c r="C62" s="14" t="s">
+      <c r="C68" s="14" t="s">
         <v>56</v>
-      </c>
-      <c r="D62" s="13"/>
-      <c r="E62" s="13"/>
-    </row>
-    <row r="63" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A63" s="21" t="s">
-        <v>87</v>
-      </c>
-      <c r="B63" s="15" t="s">
-        <v>17</v>
-      </c>
-      <c r="C63" s="15" t="s">
-        <v>58</v>
-      </c>
-      <c r="D63" s="6" t="s">
-        <v>22</v>
-      </c>
-      <c r="E63" s="6" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="64" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A64" s="21" t="s">
-        <v>88</v>
-      </c>
-      <c r="B64" s="15" t="s">
-        <v>18</v>
-      </c>
-      <c r="C64" s="15" t="s">
-        <v>59</v>
-      </c>
-      <c r="D64" s="13">
-        <v>40.299999999999997</v>
-      </c>
-      <c r="E64" s="13">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="65" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A65" s="21" t="s">
-        <v>102</v>
-      </c>
-      <c r="B65" s="15" t="s">
-        <v>19</v>
-      </c>
-      <c r="C65" s="15" t="s">
-        <v>60</v>
-      </c>
-      <c r="D65" s="13">
-        <v>51.3</v>
-      </c>
-      <c r="E65" s="13">
-        <v>55.5</v>
-      </c>
-    </row>
-    <row r="66" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A66" s="21" t="s">
-        <v>89</v>
-      </c>
-      <c r="B66" s="15" t="s">
-        <v>20</v>
-      </c>
-      <c r="C66" s="15" t="s">
-        <v>61</v>
-      </c>
-      <c r="D66" s="13">
-        <v>49.5</v>
-      </c>
-      <c r="E66" s="13">
-        <v>62.5</v>
-      </c>
-    </row>
-    <row r="67" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A67" s="21" t="s">
-        <v>90</v>
-      </c>
-      <c r="B67" s="15" t="s">
-        <v>21</v>
-      </c>
-      <c r="C67" s="15" t="s">
-        <v>62</v>
-      </c>
-      <c r="D67" s="18">
-        <v>58.2</v>
-      </c>
-      <c r="E67" s="18">
-        <v>60.1</v>
-      </c>
-    </row>
-    <row r="68" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A68" s="27" t="s">
-        <v>106</v>
-      </c>
-      <c r="B68" s="14" t="s">
-        <v>23</v>
-      </c>
-      <c r="C68" s="14" t="s">
-        <v>46</v>
       </c>
       <c r="D68" s="13"/>
       <c r="E68" s="13"/>
     </row>
     <row r="69" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A69" s="1" t="s">
+      <c r="A69" s="21" t="s">
+        <v>87</v>
+      </c>
+      <c r="B69" s="15" t="s">
+        <v>17</v>
+      </c>
+      <c r="C69" s="15" t="s">
+        <v>58</v>
+      </c>
+      <c r="D69" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="E69" s="6" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="70" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A70" s="21" t="s">
+        <v>88</v>
+      </c>
+      <c r="B70" s="15" t="s">
+        <v>18</v>
+      </c>
+      <c r="C70" s="15" t="s">
+        <v>59</v>
+      </c>
+      <c r="D70" s="13">
+        <v>40.299999999999997</v>
+      </c>
+      <c r="E70" s="13">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="71" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A71" s="21" t="s">
+        <v>102</v>
+      </c>
+      <c r="B71" s="15" t="s">
+        <v>19</v>
+      </c>
+      <c r="C71" s="15" t="s">
+        <v>60</v>
+      </c>
+      <c r="D71" s="13">
+        <v>51.3</v>
+      </c>
+      <c r="E71" s="13">
+        <v>55.5</v>
+      </c>
+    </row>
+    <row r="72" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A72" s="21" t="s">
+        <v>89</v>
+      </c>
+      <c r="B72" s="15" t="s">
+        <v>20</v>
+      </c>
+      <c r="C72" s="15" t="s">
+        <v>61</v>
+      </c>
+      <c r="D72" s="13">
+        <v>49.5</v>
+      </c>
+      <c r="E72" s="13">
+        <v>62.5</v>
+      </c>
+    </row>
+    <row r="73" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A73" s="21" t="s">
+        <v>90</v>
+      </c>
+      <c r="B73" s="15" t="s">
+        <v>21</v>
+      </c>
+      <c r="C73" s="15" t="s">
+        <v>62</v>
+      </c>
+      <c r="D73" s="18">
+        <v>58.2</v>
+      </c>
+      <c r="E73" s="18">
+        <v>60.1</v>
+      </c>
+    </row>
+    <row r="74" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A74" s="27" t="s">
+        <v>106</v>
+      </c>
+      <c r="B74" s="14" t="s">
+        <v>23</v>
+      </c>
+      <c r="C74" s="14" t="s">
+        <v>46</v>
+      </c>
+      <c r="D74" s="13"/>
+      <c r="E74" s="13"/>
+    </row>
+    <row r="75" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A75" s="1" t="s">
         <v>92</v>
       </c>
-      <c r="B69" s="9" t="s">
+      <c r="B75" s="9" t="s">
         <v>24</v>
       </c>
-      <c r="C69" s="9" t="s">
+      <c r="C75" s="9" t="s">
         <v>63</v>
       </c>
-      <c r="D69" s="13">
+      <c r="D75" s="13">
         <v>39</v>
       </c>
-      <c r="E69" s="13">
+      <c r="E75" s="13">
         <v>44.9</v>
       </c>
     </row>
-    <row r="70" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A70" s="1" t="s">
+    <row r="76" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A76" s="1" t="s">
         <v>93</v>
       </c>
-      <c r="B70" s="9" t="s">
+      <c r="B76" s="9" t="s">
         <v>25</v>
       </c>
-      <c r="C70" s="9" t="s">
+      <c r="C76" s="9" t="s">
         <v>64</v>
       </c>
-      <c r="D70" s="13">
+      <c r="D76" s="13">
         <v>52.6</v>
       </c>
-      <c r="E70" s="13">
+      <c r="E76" s="13">
         <v>57.7</v>
       </c>
     </row>
-    <row r="71" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A71" s="27" t="s">
+    <row r="77" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A77" s="27" t="s">
         <v>107</v>
       </c>
-      <c r="B71" s="14" t="s">
+      <c r="B77" s="14" t="s">
         <v>26</v>
       </c>
-      <c r="C71" s="14" t="s">
+      <c r="C77" s="14" t="s">
         <v>47</v>
       </c>
-      <c r="D71" s="13"/>
-      <c r="E71" s="13"/>
-    </row>
-    <row r="72" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A72" s="1" t="s">
+      <c r="D77" s="13"/>
+      <c r="E77" s="13"/>
+    </row>
+    <row r="78" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A78" s="1" t="s">
         <v>92</v>
       </c>
-      <c r="B72" s="9" t="s">
+      <c r="B78" s="9" t="s">
         <v>24</v>
       </c>
-      <c r="C72" s="9" t="s">
+      <c r="C78" s="9" t="s">
         <v>63</v>
       </c>
-      <c r="D72" s="13">
+      <c r="D78" s="13">
         <v>47.9</v>
       </c>
-      <c r="E72" s="18" t="s">
+      <c r="E78" s="18" t="s">
         <v>124</v>
       </c>
     </row>
-    <row r="73" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A73" s="1" t="s">
+    <row r="79" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A79" s="1" t="s">
         <v>93</v>
       </c>
-      <c r="B73" s="9" t="s">
+      <c r="B79" s="9" t="s">
         <v>25</v>
       </c>
-      <c r="C73" s="9" t="s">
+      <c r="C79" s="9" t="s">
         <v>64</v>
       </c>
-      <c r="D73" s="18">
+      <c r="D79" s="18">
         <v>52</v>
       </c>
-      <c r="E73" s="18">
+      <c r="E79" s="18">
         <v>55.2</v>
       </c>
     </row>
-    <row r="74" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A74" s="1" t="s">
+    <row r="80" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A80" s="1" t="s">
         <v>105</v>
       </c>
-      <c r="B74" s="9" t="s">
+      <c r="B80" s="9" t="s">
         <v>27</v>
       </c>
-      <c r="C74" s="9" t="s">
+      <c r="C80" s="9" t="s">
         <v>65</v>
       </c>
-      <c r="D74" s="13">
+      <c r="D80" s="13">
         <v>49.1</v>
       </c>
-      <c r="E74" s="18" t="s">
+      <c r="E80" s="18" t="s">
         <v>125</v>
       </c>
     </row>
-    <row r="75" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A75" s="14" t="s">
+    <row r="81" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A81" s="14" t="s">
         <v>104</v>
       </c>
-      <c r="B75" s="14" t="s">
+      <c r="B81" s="14" t="s">
         <v>53</v>
       </c>
-      <c r="C75" s="14" t="s">
+      <c r="C81" s="14" t="s">
         <v>57</v>
       </c>
-      <c r="D75" s="13"/>
-      <c r="E75" s="13"/>
-    </row>
-    <row r="76" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A76" s="24" t="s">
+      <c r="D81" s="13"/>
+      <c r="E81" s="13"/>
+    </row>
+    <row r="82" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A82" s="24" t="s">
         <v>95</v>
       </c>
-      <c r="B76" s="15" t="s">
+      <c r="B82" s="15" t="s">
         <v>28</v>
       </c>
-      <c r="C76" s="15" t="s">
+      <c r="C82" s="15" t="s">
         <v>66</v>
       </c>
-      <c r="D76" s="13">
+      <c r="D82" s="13">
         <v>50.8</v>
       </c>
-      <c r="E76" s="13">
+      <c r="E82" s="13">
         <v>57.1</v>
       </c>
     </row>
-    <row r="77" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A77" s="24" t="s">
+    <row r="83" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A83" s="24" t="s">
         <v>96</v>
       </c>
-      <c r="B77" s="15" t="s">
+      <c r="B83" s="15" t="s">
         <v>29</v>
       </c>
-      <c r="C77" s="15" t="s">
+      <c r="C83" s="15" t="s">
         <v>67</v>
       </c>
-      <c r="D77" s="13">
+      <c r="D83" s="13">
         <v>42.6</v>
       </c>
-      <c r="E77" s="13">
+      <c r="E83" s="13">
         <v>50.8</v>
       </c>
     </row>
-    <row r="78" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A78" s="24" t="s">
+    <row r="84" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A84" s="24" t="s">
         <v>97</v>
       </c>
-      <c r="B78" s="15" t="s">
+      <c r="B84" s="15" t="s">
         <v>30</v>
       </c>
-      <c r="C78" s="15" t="s">
+      <c r="C84" s="15" t="s">
         <v>68</v>
       </c>
-      <c r="D78" s="13">
+      <c r="D84" s="13">
         <v>52.1</v>
       </c>
-      <c r="E78" s="13">
+      <c r="E84" s="13">
         <v>54.3</v>
       </c>
     </row>
-    <row r="79" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A79" s="24" t="s">
+    <row r="85" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A85" s="24" t="s">
         <v>98</v>
       </c>
-      <c r="B79" s="15" t="s">
+      <c r="B85" s="15" t="s">
         <v>31</v>
       </c>
-      <c r="C79" s="15" t="s">
+      <c r="C85" s="15" t="s">
         <v>69</v>
       </c>
-      <c r="D79" s="18">
+      <c r="D85" s="18">
         <v>50.1</v>
       </c>
-      <c r="E79" s="18">
+      <c r="E85" s="18">
         <v>59.2</v>
       </c>
     </row>
-    <row r="80" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A80" s="26" t="s">
+    <row r="86" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A86" s="26" t="s">
         <v>99</v>
       </c>
-      <c r="B80" s="16" t="s">
+      <c r="B86" s="16" t="s">
         <v>32</v>
       </c>
-      <c r="C80" s="16" t="s">
+      <c r="C86" s="16" t="s">
         <v>70</v>
       </c>
-      <c r="D80" s="7">
+      <c r="D86" s="7">
         <v>64.400000000000006</v>
       </c>
-      <c r="E80" s="7">
+      <c r="E86" s="7">
         <v>65.5</v>
       </c>
     </row>
-    <row r="81" spans="1:4" ht="26.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A81" s="17" t="s">
+    <row r="87" spans="1:5" ht="26.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A87" s="17" t="s">
         <v>118</v>
       </c>
-      <c r="B81" s="17" t="s">
+      <c r="B87" s="17" t="s">
         <v>119</v>
       </c>
-      <c r="C81" s="17" t="s">
-        <v>128</v>
-      </c>
-      <c r="D81" s="1"/>
-    </row>
-    <row r="82" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="B82" s="9"/>
-      <c r="C82" s="9"/>
-    </row>
-    <row r="83" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="B83" s="9"/>
-      <c r="C83" s="9"/>
-    </row>
-    <row r="84" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="B84" s="9"/>
-      <c r="C84" s="9"/>
-    </row>
-    <row r="85" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="B85" s="9"/>
-      <c r="C85" s="9"/>
-    </row>
-    <row r="86" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="B86" s="9"/>
-      <c r="C86" s="9"/>
-    </row>
-    <row r="87" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="B87" s="9"/>
-      <c r="C87" s="9"/>
-    </row>
-    <row r="88" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="C87" s="17" t="s">
+        <v>137</v>
+      </c>
+      <c r="D87" s="1"/>
+    </row>
+    <row r="88" spans="1:5" x14ac:dyDescent="0.25">
       <c r="B88" s="9"/>
       <c r="C88" s="9"/>
     </row>
-    <row r="89" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="89" spans="1:5" x14ac:dyDescent="0.25">
       <c r="B89" s="9"/>
       <c r="C89" s="9"/>
     </row>
-    <row r="90" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="90" spans="1:5" x14ac:dyDescent="0.25">
       <c r="B90" s="9"/>
       <c r="C90" s="9"/>
     </row>
-    <row r="91" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="91" spans="1:5" x14ac:dyDescent="0.25">
       <c r="B91" s="9"/>
       <c r="C91" s="9"/>
     </row>
-    <row r="92" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="92" spans="1:5" x14ac:dyDescent="0.25">
       <c r="B92" s="9"/>
       <c r="C92" s="9"/>
     </row>
-    <row r="93" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="93" spans="1:5" x14ac:dyDescent="0.25">
       <c r="B93" s="9"/>
       <c r="C93" s="9"/>
     </row>
-    <row r="94" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="94" spans="1:5" x14ac:dyDescent="0.25">
       <c r="B94" s="9"/>
       <c r="C94" s="9"/>
     </row>
-    <row r="95" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="95" spans="1:5" x14ac:dyDescent="0.25">
       <c r="B95" s="9"/>
       <c r="C95" s="9"/>
     </row>
-    <row r="96" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="96" spans="1:5" x14ac:dyDescent="0.25">
       <c r="B96" s="9"/>
       <c r="C96" s="9"/>
     </row>
@@ -2928,6 +3027,30 @@
     <row r="240" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B240" s="9"/>
       <c r="C240" s="9"/>
+    </row>
+    <row r="241" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B241" s="9"/>
+      <c r="C241" s="9"/>
+    </row>
+    <row r="242" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B242" s="9"/>
+      <c r="C242" s="9"/>
+    </row>
+    <row r="243" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B243" s="9"/>
+      <c r="C243" s="9"/>
+    </row>
+    <row r="244" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B244" s="9"/>
+      <c r="C244" s="9"/>
+    </row>
+    <row r="245" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B245" s="9"/>
+      <c r="C245" s="9"/>
+    </row>
+    <row r="246" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B246" s="9"/>
+      <c r="C246" s="9"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>